<commit_message>
Add stock tracking UI, material templates update, and warning logic integration
- app.py: Added /stock route for inventory management, integrated stock warning checks into calculation routes, implemented atomic file operations for materials database
- db.py: Extended schema with stock_moves table for transaction logging, added migration support for new stock-related columns in postings table
- data/materials.xlsx: Updated template to include stock unit, remaining quantity, kg per unit, and invoice reference fields
- templates/stock.html: Created new UI page for viewing and editing material stock levels and units
- .gitignore: Cleaned up ignore rules to properly exclude Python cache files
</commit_message>
<xml_diff>
--- a/data/materials.xlsx
+++ b/data/materials.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Материалы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,26 @@
           <t>Примечание</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Единица учёта</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Остаток на складе</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Кг на 1 единицу учёта</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Накладная</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,7 +505,6 @@
       <c r="F2" t="n">
         <v>85</v>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,7 +533,6 @@
       <c r="F3" t="n">
         <v>85</v>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -543,7 +561,6 @@
       <c r="F4" t="n">
         <v>70</v>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -572,7 +589,6 @@
       <c r="F5" t="n">
         <v>75</v>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -601,7 +617,6 @@
       <c r="F6" t="n">
         <v>70</v>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -633,7 +648,6 @@
       <c r="G7" t="n">
         <v>4.62</v>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -646,7 +660,6 @@
           <t>Капролон</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>50</t>
@@ -658,7 +671,6 @@
       <c r="F8" t="n">
         <v>400</v>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -671,7 +683,6 @@
           <t>Текстолит</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>10х500х500</t>
@@ -683,7 +694,6 @@
       <c r="F9" t="n">
         <v>600</v>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>